<commit_message>
📊 TABLE2: Add training time column to detection performance table
Changes:
- Added detection_training_times dict (12 actual values from results.csv)
- Changed table structure from 4 to 5 metrics per YOLO model
- Removed "Medium (20.1M params)" from headers → just model names
- Added "Time (min)" as 5th metric column after Recall
- Updated column widths (13 → 15 metric columns)
- Regenerated Table2_Detection_Performance.xlsx

Training times extracted from:
- results/optA_20251016_200330/experiments/.../det_*/results.csv
- Format: Last epoch cumulative seconds → minutes

Structure: 4 datasets × 3 YOLO × 5 metrics = 4 rows × 16 columns
Metrics: mAP@50, mAP@50-95, Precision, Recall, Time

🤖 Generated with Claude Code

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/luaran/templates/tables/Table2_Detection_Performance.xlsx
+++ b/luaran/templates/tables/Table2_Detection_Performance.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -473,6 +473,9 @@
     <col width="11" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
     <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
@@ -483,20 +486,17 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>YOLOv10
-Medium (20.1M params)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>YOLOv11
-Medium (20.1M params)</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>YOLOv12
-Medium (20.1M params)</t>
+          <t>YOLOv10</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>YOLOv11</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>YOLOv12</t>
         </is>
       </c>
     </row>
@@ -528,50 +528,68 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
+          <t>Time
+(min)</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
           <t>mAP@50
 (%)</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>mAP@50-95
 (%)</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Precision
 (%)</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>Recall
 (%)</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>Time
+(min)</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>mAP@50
 (%)</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>mAP@50-95
 (%)</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>Precision
 (%)</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>Recall
 (%)</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>Time
+(min)</t>
         </is>
       </c>
     </row>
@@ -594,28 +612,37 @@
         <v>92.22</v>
       </c>
       <c r="F3" s="5" t="n">
+        <v>6.33</v>
+      </c>
+      <c r="G3" s="5" t="n">
         <v>94.98999999999999</v>
       </c>
-      <c r="G3" s="5" t="n">
+      <c r="H3" s="5" t="n">
         <v>77.76000000000001</v>
       </c>
-      <c r="H3" s="5" t="n">
+      <c r="I3" s="5" t="n">
         <v>91.91</v>
       </c>
-      <c r="I3" s="5" t="n">
+      <c r="J3" s="5" t="n">
         <v>91.11</v>
       </c>
-      <c r="J3" s="5" t="n">
+      <c r="K3" s="5" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="L3" s="5" t="n">
         <v>94.40000000000001</v>
       </c>
-      <c r="K3" s="5" t="n">
+      <c r="M3" s="5" t="n">
         <v>78.20999999999999</v>
       </c>
-      <c r="L3" s="5" t="n">
+      <c r="N3" s="5" t="n">
         <v>92.2</v>
       </c>
-      <c r="M3" s="5" t="n">
+      <c r="O3" s="5" t="n">
         <v>86.67</v>
+      </c>
+      <c r="P3" s="5" t="n">
+        <v>7.55</v>
       </c>
     </row>
     <row r="4" ht="25" customHeight="1">
@@ -637,28 +664,37 @@
         <v>90.73</v>
       </c>
       <c r="F4" s="5" t="n">
+        <v>4.42</v>
+      </c>
+      <c r="G4" s="5" t="n">
         <v>92.56999999999999</v>
       </c>
-      <c r="G4" s="5" t="n">
+      <c r="H4" s="5" t="n">
         <v>62.17</v>
       </c>
-      <c r="H4" s="5" t="n">
+      <c r="I4" s="5" t="n">
         <v>86.52</v>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="J4" s="5" t="n">
         <v>91.88</v>
       </c>
-      <c r="J4" s="5" t="n">
+      <c r="K4" s="5" t="n">
+        <v>4.78</v>
+      </c>
+      <c r="L4" s="5" t="n">
         <v>92.72</v>
       </c>
-      <c r="K4" s="5" t="n">
+      <c r="M4" s="5" t="n">
         <v>62.25</v>
       </c>
-      <c r="L4" s="5" t="n">
+      <c r="N4" s="5" t="n">
         <v>88.98999999999999</v>
       </c>
-      <c r="M4" s="5" t="n">
+      <c r="O4" s="5" t="n">
         <v>89.28</v>
+      </c>
+      <c r="P4" s="5" t="n">
+        <v>4.71</v>
       </c>
     </row>
     <row r="5" ht="25" customHeight="1">
@@ -680,28 +716,37 @@
         <v>93.12</v>
       </c>
       <c r="F5" s="5" t="n">
+        <v>3.82</v>
+      </c>
+      <c r="G5" s="5" t="n">
         <v>94.48</v>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="H5" s="5" t="n">
         <v>60.34</v>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="I5" s="5" t="n">
         <v>93.15000000000001</v>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="J5" s="5" t="n">
         <v>88.36</v>
       </c>
-      <c r="J5" s="5" t="n">
+      <c r="K5" s="5" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="L5" s="5" t="n">
         <v>96.27</v>
       </c>
-      <c r="K5" s="5" t="n">
+      <c r="M5" s="5" t="n">
         <v>61.53</v>
       </c>
-      <c r="L5" s="5" t="n">
+      <c r="N5" s="5" t="n">
         <v>92.91</v>
       </c>
-      <c r="M5" s="5" t="n">
+      <c r="O5" s="5" t="n">
         <v>92.59</v>
+      </c>
+      <c r="P5" s="5" t="n">
+        <v>5.79</v>
       </c>
     </row>
     <row r="6" ht="25" customHeight="1">
@@ -723,35 +768,44 @@
         <v>71.05</v>
       </c>
       <c r="F6" s="5" t="n">
+        <v>9.890000000000001</v>
+      </c>
+      <c r="G6" s="5" t="n">
         <v>72.91</v>
       </c>
-      <c r="G6" s="5" t="n">
+      <c r="H6" s="5" t="n">
         <v>57.71</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="I6" s="5" t="n">
         <v>68.58</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="J6" s="5" t="n">
         <v>75.7</v>
       </c>
-      <c r="J6" s="5" t="n">
+      <c r="K6" s="5" t="n">
+        <v>9.130000000000001</v>
+      </c>
+      <c r="L6" s="5" t="n">
         <v>71.12</v>
       </c>
-      <c r="K6" s="5" t="n">
+      <c r="M6" s="5" t="n">
         <v>56.93</v>
       </c>
-      <c r="L6" s="5" t="n">
+      <c r="N6" s="5" t="n">
         <v>65.92</v>
       </c>
-      <c r="M6" s="5" t="n">
+      <c r="O6" s="5" t="n">
         <v>75.18000000000001</v>
+      </c>
+      <c r="P6" s="5" t="n">
+        <v>13.67</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="J1:M1"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="L1:P1"/>
+    <mergeCell ref="B1:F1"/>
+    <mergeCell ref="G1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>